<commit_message>
Atualiza planilha TRANSFERENCIA (run automatico)
</commit_message>
<xml_diff>
--- a/output/TRANSFERENCIA_atual.xlsx
+++ b/output/TRANSFERENCIA_atual.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxa de Transferência" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Taxa de Transferência" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxa de Transferência'!$A$1:$E$20</definedName>

</xml_diff>

<commit_message>
Corrige planilha TRANSFERENCIA (reenvio manual, dado de 06h saiu zerado)
</commit_message>
<xml_diff>
--- a/output/TRANSFERENCIA_atual.xlsx
+++ b/output/TRANSFERENCIA_atual.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Taxa de Transferência" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxa de Transferência" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxa de Transferência'!$A$1:$F$34</definedName>
@@ -484,15 +484,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>3744</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>3678</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2" t="n"/>
+        <v>66</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.9823999999999999</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -506,15 +508,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1863</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1853</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.9945999999999999</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -528,15 +532,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1144</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1137</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.9939</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -550,15 +556,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>459</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>443</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2" t="n"/>
+        <v>16</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.9651000000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -572,10 +580,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9006</v>
+        <v>20520</v>
       </c>
       <c r="D6" t="n">
-        <v>9006</v>
+        <v>20520</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -596,15 +604,17 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>18492</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>13851</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2" t="n"/>
+        <v>4641</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.7490000000000001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -618,16 +628,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5872</v>
+        <v>7613</v>
       </c>
       <c r="D8" t="n">
-        <v>2867</v>
+        <v>4595</v>
       </c>
       <c r="E8" t="n">
-        <v>3005</v>
+        <v>3018</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.4882</v>
+        <v>0.6036</v>
       </c>
     </row>
     <row r="9">
@@ -642,15 +652,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>20210</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>19286</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="2" t="n"/>
+        <v>924</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0.9543</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -686,10 +698,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>67187</v>
+        <v>127528</v>
       </c>
       <c r="D11" t="n">
-        <v>67187</v>
+        <v>127528</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -710,15 +722,17 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>2566</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>2398</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="2" t="n"/>
+        <v>168</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.9345</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -732,16 +746,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2088</v>
+        <v>4027</v>
       </c>
       <c r="D13" t="n">
-        <v>2088</v>
+        <v>4026</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
     </row>
     <row r="14">
@@ -756,15 +770,17 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>5207</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>5205</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0.9995999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -800,15 +816,17 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>595</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>585</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="2" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>0.9832</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -822,10 +840,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2015</v>
+        <v>5556</v>
       </c>
       <c r="D17" t="n">
-        <v>2015</v>
+        <v>5556</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -868,15 +886,17 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1342</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1336</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="2" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.9954999999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -890,15 +910,17 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>9466</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>9298</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="2" t="n"/>
+        <v>168</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>0.9823000000000001</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -934,15 +956,17 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>2831</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>2780</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="2" t="n"/>
+        <v>51</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0.982</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -956,15 +980,17 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>30099</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>29250</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="2" t="n"/>
+        <v>849</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.9718000000000001</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1000,15 +1026,17 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>51339</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>50410</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="2" t="n"/>
+        <v>929</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0.9819</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1022,16 +1050,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>12356</v>
+        <v>22446</v>
       </c>
       <c r="D26" t="n">
-        <v>5880</v>
+        <v>12693</v>
       </c>
       <c r="E26" t="n">
-        <v>6476</v>
+        <v>9753</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.4759</v>
+        <v>0.5655</v>
       </c>
     </row>
     <row r="27">
@@ -1046,16 +1074,16 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>11981</v>
+        <v>22818</v>
       </c>
       <c r="D27" t="n">
-        <v>6538</v>
+        <v>15173</v>
       </c>
       <c r="E27" t="n">
-        <v>5443</v>
+        <v>7645</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.5457</v>
+        <v>0.665</v>
       </c>
     </row>
     <row r="28">
@@ -1094,16 +1122,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4108</v>
+        <v>8850</v>
       </c>
       <c r="D29" t="n">
-        <v>2516</v>
+        <v>5450</v>
       </c>
       <c r="E29" t="n">
-        <v>1592</v>
+        <v>3400</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.6125</v>
+        <v>0.6158</v>
       </c>
     </row>
     <row r="30">
@@ -1118,15 +1146,17 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>1128</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1112</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="2" t="n"/>
+        <v>16</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0.9858</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1162,15 +1192,17 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>10073</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>9975</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="2" t="n"/>
+        <v>98</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0.9903</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1184,15 +1216,17 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>25750</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>25239</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="2" t="n"/>
+        <v>511</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0.9802</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">

</xml_diff>